<commit_message>
publish live hog price report 2026-07-23
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-22</t>
+          <t>越南生猪价格省级明细｜2026-07-23</t>
         </is>
       </c>
     </row>
@@ -585,14 +585,14 @@
         <v>65000</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>67000</v>
+        <v>66000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>66000</v>
+        <v>65733</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>太原 -1,000、莱州 -1,000、山罗 -1,000</t>
+          <t>河内 -1,000、宁平 -1,000、老街 -1,000、兴安 -1,000</t>
         </is>
       </c>
     </row>
@@ -609,14 +609,14 @@
         <v>62000</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>65000</v>
+        <v>64000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>63545</v>
+        <v>63364</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>总体稳定</t>
+          <t>清化 -1,000、乂安 -1,000</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-227-tiep-da-giam-tai-mien-bac-202672264651882.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-237-tiep-tuc-di-xuong-66000-dongkg-la-muc-giao-dich-cao-nhat-duoc-ghi-nhan-20267237017809.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-22</t>
+          <t>越南生猪价格｜北部｜2026-07-23</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,10 @@
       <c r="C7" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -860,12 +858,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>67000</v>
-      </c>
-      <c r="D11" s="8" t="n"/>
+        <v>66000</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -902,12 +902,14 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D13" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -923,12 +925,14 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D14" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -946,12 +950,10 @@
       <c r="C15" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D15" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1011,12 +1013,10 @@
       <c r="C18" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D18" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D18" s="8" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1032,12 +1032,14 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>67000</v>
-      </c>
-      <c r="D19" s="8" t="n"/>
+        <v>66000</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1071,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-22</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-23</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1121,14 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D5" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1144,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1372,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-22</t>
+          <t>越南生猪价格｜南部｜2026-07-23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-24
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -144,10 +144,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-24</t>
+          <t>越南生猪价格省级明细｜2026-07-25</t>
         </is>
       </c>
     </row>
@@ -582,17 +582,17 @@
         <v>15</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>65000</v>
+        <v>64000</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>66000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>65733</v>
+        <v>65200</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>河内 -1,000、宁平 -1,000、老街 -1,000、兴安 -1,000</t>
+          <t>宣光 -1,000、谅山 -1,000、广宁 -1,000、北宁 -1,000、宁平 -1,000、老街 -1,000、莱州 -1,000、富寿 -1,000</t>
         </is>
       </c>
     </row>
@@ -612,11 +612,11 @@
         <v>64000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>63364</v>
+        <v>63091</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>清化 -1,000、乂安 -1,000</t>
+          <t>清化 -1,000、乂安 -1,000、河静 -1,000</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-237-tiep-tuc-di-xuong-66000-dongkg-la-muc-giao-dich-cao-nhat-duoc-ghi-nhan-20267237017809.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-247-tiep-da-giam-mien-bac-xuong-duoi-65000-dongkg-202672471538796.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-24</t>
+          <t>越南生猪价格｜北部｜2026-07-25</t>
         </is>
       </c>
     </row>
@@ -732,12 +732,14 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D5" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -755,7 +757,7 @@
       <c r="C6" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -776,7 +778,7 @@
       <c r="C7" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -795,12 +797,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D8" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -816,12 +820,14 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D9" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D9" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -837,12 +843,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -860,12 +868,10 @@
       <c r="C11" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="9" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -883,7 +889,7 @@
       <c r="C12" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -902,9 +908,9 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D13" s="9" t="n">
+        <v>64000</v>
+      </c>
+      <c r="D13" s="8" t="n">
         <v>-1000</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -925,9 +931,9 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D14" s="9" t="n">
+        <v>64000</v>
+      </c>
+      <c r="D14" s="8" t="n">
         <v>-1000</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -948,12 +954,14 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D15" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -971,7 +979,7 @@
       <c r="C16" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D16" s="8" t="n"/>
+      <c r="D16" s="9" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -990,12 +998,14 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D17" s="8" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1023,7 @@
       <c r="C18" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D18" s="8" t="n"/>
+      <c r="D18" s="9" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1034,12 +1044,10 @@
       <c r="C19" s="6" t="n">
         <v>66000</v>
       </c>
-      <c r="D19" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D19" s="9" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1079,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-24</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-25</t>
         </is>
       </c>
     </row>
@@ -1121,9 +1129,9 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D5" s="9" t="n">
+        <v>63000</v>
+      </c>
+      <c r="D5" s="8" t="n">
         <v>-1000</v>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -1144,9 +1152,9 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D6" s="9" t="n">
+        <v>63000</v>
+      </c>
+      <c r="D6" s="8" t="n">
         <v>-1000</v>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -1167,12 +1175,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D7" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1200,7 @@
       <c r="C8" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1211,7 +1221,7 @@
       <c r="C9" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1232,7 +1242,7 @@
       <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1253,7 +1263,7 @@
       <c r="C11" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1274,7 +1284,7 @@
       <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1295,7 +1305,7 @@
       <c r="C13" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D13" s="8" t="n"/>
+      <c r="D13" s="9" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1316,7 +1326,7 @@
       <c r="C14" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D14" s="8" t="n"/>
+      <c r="D14" s="9" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1337,7 +1347,7 @@
       <c r="C15" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1372,7 +1382,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-24</t>
+          <t>越南生猪价格｜南部｜2026-07-25</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1434,7 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="9" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1445,7 +1455,7 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1466,7 +1476,7 @@
       <c r="C7" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1487,7 +1497,7 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1508,7 +1518,7 @@
       <c r="C9" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1529,7 +1539,7 @@
       <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1550,7 +1560,7 @@
       <c r="C11" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1571,7 +1581,7 @@
       <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-25
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -144,10 +144,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-25</t>
+          <t>越南生猪价格省级明细｜2026-07-26</t>
         </is>
       </c>
     </row>
@@ -582,17 +582,17 @@
         <v>15</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>64000</v>
+        <v>63000</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>66000</v>
+        <v>65000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>65200</v>
+        <v>64733</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>宣光 -1,000、谅山 -1,000、广宁 -1,000、北宁 -1,000、宁平 -1,000、老街 -1,000、莱州 -1,000、富寿 -1,000</t>
+          <t>高平 -1,000、太原 -1,000、河内 -1,000、海防 -1,000、宁平 -1,000、奠边 -1,000、兴安 -1,000</t>
         </is>
       </c>
     </row>
@@ -609,14 +609,14 @@
         <v>62000</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>64000</v>
+        <v>63000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>63091</v>
+        <v>62909</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>清化 -1,000、乂安 -1,000、河静 -1,000</t>
+          <t>广治 -1,000、顺化 -1,000</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-247-tiep-da-giam-mien-bac-xuong-duoi-65000-dongkg-202672471538796.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-257-tiep-tuc-di-xuong-muc-63000-dongkg-duoc-ghi-nhan-tai-mien-bac-20267257330339.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-25</t>
+          <t>越南生猪价格｜北部｜2026-07-26</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,10 @@
       <c r="C5" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -755,12 +753,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D6" s="9" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D7" s="9" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -799,12 +801,10 @@
       <c r="C8" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -822,12 +822,10 @@
       <c r="C9" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D9" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -845,12 +843,10 @@
       <c r="C10" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -866,12 +862,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D11" s="9" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -887,12 +885,14 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D12" s="9" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -908,9 +908,9 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D13" s="8" t="n">
+        <v>63000</v>
+      </c>
+      <c r="D13" s="9" t="n">
         <v>-1000</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -933,12 +933,10 @@
       <c r="C14" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D14" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -956,12 +954,10 @@
       <c r="C15" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D15" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -977,12 +973,14 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D16" s="9" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1000,12 +998,10 @@
       <c r="C17" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D17" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1019,7 @@
       <c r="C18" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D18" s="9" t="n"/>
+      <c r="D18" s="8" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1042,12 +1038,14 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>66000</v>
-      </c>
-      <c r="D19" s="9" t="n"/>
+        <v>65000</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1077,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-25</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-26</t>
         </is>
       </c>
     </row>
@@ -1131,12 +1129,10 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1154,12 +1150,10 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1177,12 +1171,10 @@
       <c r="C7" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1198,12 +1190,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D8" s="9" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1219,12 +1213,14 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D9" s="9" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1238,7 @@
       <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1263,7 +1259,7 @@
       <c r="C11" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1284,7 +1280,7 @@
       <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1305,7 +1301,7 @@
       <c r="C13" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D13" s="9" t="n"/>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1326,7 +1322,7 @@
       <c r="C14" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D14" s="9" t="n"/>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1347,7 +1343,7 @@
       <c r="C15" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D15" s="9" t="n"/>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1382,7 +1378,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-25</t>
+          <t>越南生猪价格｜南部｜2026-07-26</t>
         </is>
       </c>
     </row>
@@ -1434,7 +1430,7 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1455,7 +1451,7 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1476,7 +1472,7 @@
       <c r="C7" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1497,7 +1493,7 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="9" t="n"/>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1518,7 +1514,7 @@
       <c r="C9" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1539,7 +1535,7 @@
       <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1560,7 +1556,7 @@
       <c r="C11" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1581,7 +1577,7 @@
       <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-26
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -57,7 +57,7 @@
       <color rgb="006B4C00"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,11 +89,6 @@
         <fgColor rgb="00FFF4CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -145,9 +140,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +521,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-26</t>
+          <t>越南生猪价格省级明细｜2026-07-27</t>
         </is>
       </c>
     </row>
@@ -592,7 +584,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>高平 -1,000、太原 -1,000、河内 -1,000、海防 -1,000、宁平 -1,000、奠边 -1,000、兴安 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
@@ -616,7 +608,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广治 -1,000、顺化 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
@@ -647,7 +639,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-257-tiep-tuc-di-xuong-muc-63000-dongkg-duoc-ghi-nhan-tai-mien-bac-20267257330339.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-267-lien-tuc-giam-trong-tuan-qua-thi-truong-giao-dich-trong-khoang-62000-65000-dongkg-2026726101222164.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +674,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-26</t>
+          <t>越南生猪价格｜北部｜2026-07-27</t>
         </is>
       </c>
     </row>
@@ -755,12 +747,10 @@
       <c r="C6" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -778,12 +768,10 @@
       <c r="C7" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -864,12 +852,10 @@
       <c r="C11" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -887,12 +873,10 @@
       <c r="C12" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -910,12 +894,10 @@
       <c r="C13" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D13" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -975,12 +957,10 @@
       <c r="C16" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D16" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1020,10 @@
       <c r="C19" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D19" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D19" s="8" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1055,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-26</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-27</t>
         </is>
       </c>
     </row>
@@ -1192,12 +1170,10 @@
       <c r="C8" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1215,12 +1191,10 @@
       <c r="C9" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1352,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-26</t>
+          <t>越南生猪价格｜南部｜2026-07-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-27
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -57,7 +57,7 @@
       <color rgb="006B4C00"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +89,11 @@
         <fgColor rgb="00FFF4CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -116,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -137,6 +142,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -521,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-27</t>
+          <t>越南生猪价格省级明细｜2026-07-28</t>
         </is>
       </c>
     </row>
@@ -580,11 +588,11 @@
         <v>65000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>64733</v>
+        <v>64333</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>总体稳定</t>
+          <t>宣光 -1,000、高平 -1,000、谅山 -1,000、奠边 -1,000、富寿 -1,000、山罗 -1,000</t>
         </is>
       </c>
     </row>
@@ -604,11 +612,11 @@
         <v>63000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>62909</v>
+        <v>62545</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>总体稳定</t>
+          <t>岘港 -1,000、广义 -1,000、得乐 -1,000、林同 -1,000</t>
         </is>
       </c>
     </row>
@@ -622,24 +630,24 @@
         <v>8</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>62000</v>
+        <v>61000</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>63000</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>62625</v>
+        <v>62000</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>总体稳定</t>
+          <t>西宁 -1,000、同塔 -1,000、胡志明市 -1,000、永隆 -1,000、芹苴 -1,000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-267-lien-tuc-giam-trong-tuan-qua-thi-truong-giao-dich-trong-khoang-62000-65000-dongkg-2026726101222164.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-277-ba-mien-giu-da-giam-co-noi-xuong-muc-61000-dongkg-20267277146751.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -674,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-27</t>
+          <t>越南生猪价格｜北部｜2026-07-28</t>
         </is>
       </c>
     </row>
@@ -724,12 +732,14 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D5" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -745,12 +755,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -768,7 +780,7 @@
       <c r="C7" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -787,12 +799,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D8" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -810,7 +824,7 @@
       <c r="C9" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -831,7 +845,7 @@
       <c r="C10" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -852,7 +866,7 @@
       <c r="C11" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -873,7 +887,7 @@
       <c r="C12" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -894,7 +908,7 @@
       <c r="C13" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D13" s="8" t="n"/>
+      <c r="D13" s="9" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -915,7 +929,7 @@
       <c r="C14" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D14" s="8" t="n"/>
+      <c r="D14" s="9" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -936,7 +950,7 @@
       <c r="C15" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -955,12 +969,14 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D16" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -976,12 +992,14 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D17" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D17" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -997,12 +1015,14 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D18" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D18" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1040,7 @@
       <c r="C19" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D19" s="8" t="n"/>
+      <c r="D19" s="9" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1055,7 +1075,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-27</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1127,7 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="9" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1128,7 +1148,7 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1149,7 +1169,7 @@
       <c r="C7" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1170,7 +1190,7 @@
       <c r="C8" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1191,7 +1211,7 @@
       <c r="C9" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1210,12 +1230,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1231,12 +1253,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D11" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1278,7 @@
       <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1273,12 +1297,14 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D13" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D13" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1322,7 @@
       <c r="C14" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D14" s="8" t="n"/>
+      <c r="D14" s="9" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1315,12 +1341,14 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D15" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1352,7 +1380,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-27</t>
+          <t>越南生猪价格｜南部｜2026-07-28</t>
         </is>
       </c>
     </row>
@@ -1404,7 +1432,7 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="9" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1423,12 +1451,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D6" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1444,12 +1474,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D7" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D7" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1499,7 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1488,7 +1520,7 @@
       <c r="C9" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1507,12 +1539,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D10" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1528,12 +1562,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D11" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1549,12 +1585,14 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D12" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-28
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -144,10 +144,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-28</t>
+          <t>越南生猪价格省级明细｜2026-07-29</t>
         </is>
       </c>
     </row>
@@ -588,11 +588,11 @@
         <v>65000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>64333</v>
+        <v>64200</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>宣光 -1,000、高平 -1,000、谅山 -1,000、奠边 -1,000、富寿 -1,000、山罗 -1,000</t>
+          <t>太原 -1,000、广宁 -1,000</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
         <v>11</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>62000</v>
+        <v>61000</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>63000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>62545</v>
+        <v>62182</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>岘港 -1,000、广义 -1,000、得乐 -1,000、林同 -1,000</t>
+          <t>广治 -1,000、顺化 -1,000、嘉莱 -1,000、得乐 -1,000</t>
         </is>
       </c>
     </row>
@@ -633,21 +633,21 @@
         <v>61000</v>
       </c>
       <c r="D7" s="6" t="n">
-        <v>63000</v>
+        <v>62000</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>62000</v>
+        <v>61750</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>西宁 -1,000、同塔 -1,000、胡志明市 -1,000、永隆 -1,000、芹苴 -1,000</t>
+          <t>同奈 -1,000、金瓯 -1,000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-277-ba-mien-giu-da-giam-co-noi-xuong-muc-61000-dongkg-20267277146751.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-287-them-hai-tinh-giao-dich-o-muc-61000-dongkg-2026728719236.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-28</t>
+          <t>越南生猪价格｜北部｜2026-07-29</t>
         </is>
       </c>
     </row>
@@ -734,12 +734,10 @@
       <c r="C5" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -757,12 +755,10 @@
       <c r="C6" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -778,12 +774,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D7" s="9" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -801,12 +799,10 @@
       <c r="C8" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -822,12 +818,14 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D9" s="9" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -845,7 +843,7 @@
       <c r="C10" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -866,7 +864,7 @@
       <c r="C11" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -887,7 +885,7 @@
       <c r="C12" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -908,7 +906,7 @@
       <c r="C13" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D13" s="9" t="n"/>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -929,7 +927,7 @@
       <c r="C14" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D14" s="9" t="n"/>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -950,7 +948,7 @@
       <c r="C15" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D15" s="9" t="n"/>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -971,12 +969,10 @@
       <c r="C16" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D16" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -994,12 +990,10 @@
       <c r="C17" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D17" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1017,12 +1011,10 @@
       <c r="C18" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D18" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D18" s="8" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1032,7 @@
       <c r="C19" s="6" t="n">
         <v>65000</v>
       </c>
-      <c r="D19" s="9" t="n"/>
+      <c r="D19" s="8" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1075,7 +1067,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-28</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-29</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1119,7 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1148,7 +1140,7 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1169,7 +1161,7 @@
       <c r="C7" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1188,12 +1180,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D8" s="9" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1209,12 +1203,14 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D9" s="9" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1232,12 +1228,10 @@
       <c r="C10" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1255,12 +1249,10 @@
       <c r="C11" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D11" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1268,14 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D12" s="9" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1297,9 +1291,9 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D13" s="8" t="n">
+        <v>61000</v>
+      </c>
+      <c r="D13" s="9" t="n">
         <v>-1000</v>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -1322,7 +1316,7 @@
       <c r="C14" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D14" s="9" t="n"/>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1343,12 +1337,10 @@
       <c r="C15" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D15" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1372,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-28</t>
+          <t>越南生猪价格｜南部｜2026-07-29</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1422,14 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D5" s="9" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1453,12 +1447,10 @@
       <c r="C6" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D6" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1468,10 @@
       <c r="C7" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D7" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1499,7 +1489,7 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="9" t="n"/>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1518,12 +1508,14 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D9" s="9" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1541,12 +1533,10 @@
       <c r="C10" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D10" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1564,12 +1554,10 @@
       <c r="C11" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D11" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1587,12 +1575,10 @@
       <c r="C12" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D12" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-29
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-29</t>
+          <t>越南生猪价格省级明细｜2026-07-30</t>
         </is>
       </c>
     </row>
@@ -588,11 +588,11 @@
         <v>65000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>64200</v>
+        <v>64000</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>太原 -1,000、广宁 -1,000</t>
+          <t>北宁 -1,000、河内 -1,000、海防 -1,000</t>
         </is>
       </c>
     </row>
@@ -612,11 +612,11 @@
         <v>63000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>62182</v>
+        <v>61909</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广治 -1,000、顺化 -1,000、嘉莱 -1,000、得乐 -1,000</t>
+          <t>顺化 -1,000、岘港 -1,000、庆和 -1,000</t>
         </is>
       </c>
     </row>
@@ -630,24 +630,24 @@
         <v>8</v>
       </c>
       <c r="C7" s="6" t="n">
-        <v>61000</v>
+        <v>60000</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>62000</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>61750</v>
+        <v>61000</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>同奈 -1,000、金瓯 -1,000</t>
+          <t>西宁 -1,000、同塔 -1,000、安江 -1,000、金瓯 -1,000、永隆 -1,000、芹苴 -1,000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-287-them-hai-tinh-giao-dich-o-muc-61000-dongkg-2026728719236.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-297-thi-truong-ghi-nhan-muc-60000-dongkg-202672963024277.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-29</t>
+          <t>越南生猪价格｜北部｜2026-07-30</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,10 @@
       <c r="C7" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -820,12 +818,10 @@
       <c r="C9" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -841,12 +837,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -862,12 +860,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D11" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -883,12 +883,14 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D12" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1069,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-29</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-30</t>
         </is>
       </c>
     </row>
@@ -1182,12 +1184,10 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>62000</v>
+        <v>61000</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>-1000</v>
@@ -1226,12 +1226,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1270,12 +1272,10 @@
       <c r="C12" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1293,12 +1293,10 @@
       <c r="C13" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D13" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1312,14 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D14" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-29</t>
+          <t>越南生猪价格｜南部｜2026-07-30</t>
         </is>
       </c>
     </row>
@@ -1424,12 +1424,10 @@
       <c r="C5" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D5" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1445,12 +1443,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1466,12 +1466,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>61000</v>
-      </c>
-      <c r="D7" s="8" t="n"/>
+        <v>60000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1487,12 +1489,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D8" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1512,7 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>61000</v>
+        <v>60000</v>
       </c>
       <c r="D9" s="9" t="n">
         <v>-1000</v>
@@ -1552,12 +1556,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D11" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D11" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1573,12 +1579,14 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D12" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D12" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-30
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-30</t>
+          <t>越南生猪价格省级明细｜2026-07-31</t>
         </is>
       </c>
     </row>
@@ -582,17 +582,17 @@
         <v>15</v>
       </c>
       <c r="C5" s="6" t="n">
-        <v>63000</v>
+        <v>62000</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>65000</v>
+        <v>64000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>64000</v>
+        <v>63667</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>北宁 -1,000、河内 -1,000、海防 -1,000</t>
+          <t>宁平 -1,000、老街 -1,000、奠边 -1,000、富寿 -1,000、兴安 -1,000</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
         <v>11</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>61000</v>
+        <v>60000</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>63000</v>
+        <v>62000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>61909</v>
+        <v>61455</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>顺化 -1,000、岘港 -1,000、庆和 -1,000</t>
+          <t>清化 -1,000、乂安 -1,000、河静 -1,000、得乐 -1,000、林同 -1,000</t>
         </is>
       </c>
     </row>
@@ -640,14 +640,14 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>西宁 -1,000、同塔 -1,000、安江 -1,000、金瓯 -1,000、永隆 -1,000、芹苴 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-297-thi-truong-ghi-nhan-muc-60000-dongkg-202672963024277.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-307-tiep-da-giam-64000-dongkg-la-muc-giao-dich-cao-nhat-20267307167822.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-30</t>
+          <t>越南生猪价格｜北部｜2026-07-31</t>
         </is>
       </c>
     </row>
@@ -839,12 +839,10 @@
       <c r="C10" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -862,12 +860,10 @@
       <c r="C11" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -885,12 +881,10 @@
       <c r="C12" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -906,12 +900,14 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D13" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -927,12 +923,14 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D14" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -969,12 +967,14 @@
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D16" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -990,12 +990,14 @@
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D17" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1032,12 +1034,14 @@
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>65000</v>
-      </c>
-      <c r="D19" s="8" t="n"/>
+        <v>64000</v>
+      </c>
+      <c r="D19" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1073,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-30</t>
+          <t>越南生猪价格｜中部—西原｜2026-07-31</t>
         </is>
       </c>
     </row>
@@ -1119,12 +1123,14 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D5" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1140,12 +1146,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1161,12 +1169,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D7" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1215,10 @@
       <c r="C9" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1228,12 +1236,10 @@
       <c r="C10" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1291,12 +1297,14 @@
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>61000</v>
-      </c>
-      <c r="D13" s="8" t="n"/>
+        <v>60000</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1314,12 +1322,10 @@
       <c r="C14" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1335,12 +1341,14 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D15" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1380,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-30</t>
+          <t>越南生猪价格｜南部｜2026-07-31</t>
         </is>
       </c>
     </row>
@@ -1445,12 +1453,10 @@
       <c r="C6" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1468,12 +1474,10 @@
       <c r="C7" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1491,12 +1495,10 @@
       <c r="C8" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1514,12 +1516,10 @@
       <c r="C9" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1558,12 +1558,10 @@
       <c r="C11" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D11" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1581,12 +1579,10 @@
       <c r="C12" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D12" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-07-31
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-07-31</t>
+          <t>越南生猪价格省级明细｜2026-08-01</t>
         </is>
       </c>
     </row>
@@ -588,11 +588,11 @@
         <v>64000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>63667</v>
+        <v>63267</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>宁平 -1,000、老街 -1,000、奠边 -1,000、富寿 -1,000、兴安 -1,000</t>
+          <t>高平 -1,000、太原 -1,000、谅山 -1,000、广宁 -1,000、北宁 -1,000、山罗 -1,000</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>清化 -1,000、乂安 -1,000、河静 -1,000、得乐 -1,000、林同 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-307-tiep-da-giam-64000-dongkg-la-muc-giao-dich-cao-nhat-20267307167822.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-317-mien-bac-tiep-tuc-di-xuong-2026731753729.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-07-31</t>
+          <t>越南生猪价格｜北部｜2026-08-01</t>
         </is>
       </c>
     </row>
@@ -753,12 +753,14 @@
         </is>
       </c>
       <c r="C6" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D6" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -774,12 +776,14 @@
         </is>
       </c>
       <c r="C7" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D7" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -795,12 +799,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D8" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D8" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -816,12 +822,14 @@
         </is>
       </c>
       <c r="C9" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D9" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D9" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -837,12 +845,14 @@
         </is>
       </c>
       <c r="C10" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D10" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D10" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -902,12 +912,10 @@
       <c r="C13" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D13" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -925,12 +933,10 @@
       <c r="C14" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D14" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -969,12 +975,10 @@
       <c r="C16" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D16" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -992,12 +996,10 @@
       <c r="C17" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D17" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1013,12 +1015,14 @@
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D18" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D18" s="9" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1036,12 +1040,10 @@
       <c r="C19" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D19" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D19" s="8" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1075,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-07-31</t>
+          <t>越南生猪价格｜中部—西原｜2026-08-01</t>
         </is>
       </c>
     </row>
@@ -1125,12 +1127,10 @@
       <c r="C5" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D5" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1148,12 +1148,10 @@
       <c r="C6" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1171,12 +1169,10 @@
       <c r="C7" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1299,12 +1295,10 @@
       <c r="C13" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D13" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1343,12 +1337,10 @@
       <c r="C15" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D15" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1380,7 +1372,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-07-31</t>
+          <t>越南生猪价格｜南部｜2026-08-01</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
publish live hog price report 2026-08-01
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -144,10 +144,10 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +529,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-08-01</t>
+          <t>越南生猪价格省级明细｜2026-08-02</t>
         </is>
       </c>
     </row>
@@ -588,11 +588,11 @@
         <v>64000</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>63267</v>
+        <v>63000</v>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>高平 -1,000、太原 -1,000、谅山 -1,000、广宁 -1,000、北宁 -1,000、山罗 -1,000</t>
+          <t>宣光 -1,000、海防 -1,000、老街 -1,000、莱州 -1,000</t>
         </is>
       </c>
     </row>
@@ -612,11 +612,11 @@
         <v>62000</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>61455</v>
+        <v>61364</v>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>总体稳定</t>
+          <t>广义 -1,000</t>
         </is>
       </c>
     </row>
@@ -636,18 +636,18 @@
         <v>62000</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>61000</v>
+        <v>60875</v>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>总体稳定</t>
+          <t>安江 -1,000</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-317-mien-bac-tiep-tuc-di-xuong-2026731753729.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-18-bien-dong-tai-ca-ba-mien-20268173041124.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-08-01</t>
+          <t>越南生猪价格｜北部｜2026-08-02</t>
         </is>
       </c>
     </row>
@@ -732,12 +732,14 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D5" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D5" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -755,12 +757,10 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D6" s="9" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -778,12 +778,10 @@
       <c r="C7" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D7" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -801,12 +799,10 @@
       <c r="C8" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D8" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="9" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -824,12 +820,10 @@
       <c r="C9" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D9" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -847,12 +841,10 @@
       <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D10" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D10" s="9" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -870,7 +862,7 @@
       <c r="C11" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -889,12 +881,14 @@
         </is>
       </c>
       <c r="C12" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D12" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D12" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -912,7 +906,7 @@
       <c r="C13" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D13" s="8" t="n"/>
+      <c r="D13" s="9" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -931,12 +925,14 @@
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>63000</v>
-      </c>
-      <c r="D14" s="8" t="n"/>
+        <v>62000</v>
+      </c>
+      <c r="D14" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -952,12 +948,14 @@
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>64000</v>
-      </c>
-      <c r="D15" s="8" t="n"/>
+        <v>63000</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -975,7 +973,7 @@
       <c r="C16" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D16" s="8" t="n"/>
+      <c r="D16" s="9" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -996,7 +994,7 @@
       <c r="C17" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D17" s="8" t="n"/>
+      <c r="D17" s="9" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1017,12 +1015,10 @@
       <c r="C18" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D18" s="9" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D18" s="9" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1036,7 @@
       <c r="C19" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D19" s="8" t="n"/>
+      <c r="D19" s="9" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1075,7 +1071,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-08-01</t>
+          <t>越南生猪价格｜中部—西原｜2026-08-02</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1123,7 @@
       <c r="C5" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="9" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1148,7 +1144,7 @@
       <c r="C6" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1169,7 +1165,7 @@
       <c r="C7" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1190,7 +1186,7 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="8" t="n"/>
+      <c r="D8" s="9" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1211,7 +1207,7 @@
       <c r="C9" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1232,7 +1228,7 @@
       <c r="C10" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1251,12 +1247,14 @@
         </is>
       </c>
       <c r="C11" s="6" t="n">
-        <v>62000</v>
-      </c>
-      <c r="D11" s="8" t="n"/>
+        <v>61000</v>
+      </c>
+      <c r="D11" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1274,7 +1272,7 @@
       <c r="C12" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1295,7 +1293,7 @@
       <c r="C13" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D13" s="8" t="n"/>
+      <c r="D13" s="9" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1316,7 +1314,7 @@
       <c r="C14" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D14" s="8" t="n"/>
+      <c r="D14" s="9" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1337,7 +1335,7 @@
       <c r="C15" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D15" s="8" t="n"/>
+      <c r="D15" s="9" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1372,7 +1370,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-08-01</t>
+          <t>越南生猪价格｜南部｜2026-08-02</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1422,7 @@
       <c r="C5" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D5" s="8" t="n"/>
+      <c r="D5" s="9" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1445,7 +1443,7 @@
       <c r="C6" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D6" s="8" t="n"/>
+      <c r="D6" s="9" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1466,7 +1464,7 @@
       <c r="C7" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D7" s="8" t="n"/>
+      <c r="D7" s="9" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1485,12 +1483,14 @@
         </is>
       </c>
       <c r="C8" s="6" t="n">
-        <v>61000</v>
-      </c>
-      <c r="D8" s="8" t="n"/>
+        <v>60000</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>-1000</v>
+      </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>稳定</t>
+          <t>下降</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1508,7 @@
       <c r="C9" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D9" s="8" t="n"/>
+      <c r="D9" s="9" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1529,7 +1529,7 @@
       <c r="C10" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D10" s="8" t="n"/>
+      <c r="D10" s="9" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1550,7 +1550,7 @@
       <c r="C11" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D11" s="8" t="n"/>
+      <c r="D11" s="9" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1571,7 +1571,7 @@
       <c r="C12" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D12" s="8" t="n"/>
+      <c r="D12" s="9" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>

</xml_diff>

<commit_message>
publish live hog price report 2026-08-02
</commit_message>
<xml_diff>
--- a/reports/越南生猪价格省级三大区_最新.xlsx
+++ b/reports/越南生猪价格省级三大区_最新.xlsx
@@ -57,7 +57,7 @@
       <color rgb="006B4C00"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,11 +89,6 @@
         <fgColor rgb="00FFF4CC"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F5E9"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -121,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -142,9 +137,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -529,7 +521,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格省级明细｜2026-08-02</t>
+          <t>越南生猪价格省级明细｜2026-08-03</t>
         </is>
       </c>
     </row>
@@ -592,7 +584,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>宣光 -1,000、海防 -1,000、老街 -1,000、莱州 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
@@ -616,7 +608,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>广义 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
@@ -640,14 +632,14 @@
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>安江 -1,000</t>
+          <t>总体稳定</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-18-bien-dong-tai-ca-ba-mien-20268173041124.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
+          <t>来源：VietnamBiz当日活猪价格文章。原文链接：https://vietnambiz.vn/gia-heo-hoi-hom-nay-28-lien-tuc-di-xuong-thi-truong-ghi-nhan-muc-60000-dongkg-trong-tuan-qua-20268285111208.htm。使用边界：媒体报价用于行情观察，不等同于屠宰场或养殖场实际成交价；同一日数据不做跨部位或跨市场均价推断。</t>
         </is>
       </c>
     </row>
@@ -682,7 +674,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜北部｜2026-08-02</t>
+          <t>越南生猪价格｜北部｜2026-08-03</t>
         </is>
       </c>
     </row>
@@ -734,12 +726,10 @@
       <c r="C5" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D5" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -757,7 +747,7 @@
       <c r="C6" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -778,7 +768,7 @@
       <c r="C7" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -799,7 +789,7 @@
       <c r="C8" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D8" s="9" t="n"/>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -820,7 +810,7 @@
       <c r="C9" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -841,7 +831,7 @@
       <c r="C10" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -862,7 +852,7 @@
       <c r="C11" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -883,12 +873,10 @@
       <c r="C12" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D12" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -906,7 +894,7 @@
       <c r="C13" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D13" s="9" t="n"/>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -927,12 +915,10 @@
       <c r="C14" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D14" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -950,12 +936,10 @@
       <c r="C15" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D15" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -973,7 +957,7 @@
       <c r="C16" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D16" s="9" t="n"/>
+      <c r="D16" s="8" t="n"/>
       <c r="E16" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -994,7 +978,7 @@
       <c r="C17" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D17" s="9" t="n"/>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1015,7 +999,7 @@
       <c r="C18" s="6" t="n">
         <v>63000</v>
       </c>
-      <c r="D18" s="9" t="n"/>
+      <c r="D18" s="8" t="n"/>
       <c r="E18" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1036,7 +1020,7 @@
       <c r="C19" s="6" t="n">
         <v>64000</v>
       </c>
-      <c r="D19" s="9" t="n"/>
+      <c r="D19" s="8" t="n"/>
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1071,7 +1055,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜中部—西原｜2026-08-02</t>
+          <t>越南生猪价格｜中部—西原｜2026-08-03</t>
         </is>
       </c>
     </row>
@@ -1123,7 +1107,7 @@
       <c r="C5" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1144,7 +1128,7 @@
       <c r="C6" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1165,7 +1149,7 @@
       <c r="C7" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1186,7 +1170,7 @@
       <c r="C8" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D8" s="9" t="n"/>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1207,7 +1191,7 @@
       <c r="C9" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1228,7 +1212,7 @@
       <c r="C10" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1249,12 +1233,10 @@
       <c r="C11" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D11" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1272,7 +1254,7 @@
       <c r="C12" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1293,7 +1275,7 @@
       <c r="C13" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D13" s="9" t="n"/>
+      <c r="D13" s="8" t="n"/>
       <c r="E13" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1314,7 +1296,7 @@
       <c r="C14" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D14" s="9" t="n"/>
+      <c r="D14" s="8" t="n"/>
       <c r="E14" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1335,7 +1317,7 @@
       <c r="C15" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D15" s="9" t="n"/>
+      <c r="D15" s="8" t="n"/>
       <c r="E15" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1370,7 +1352,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>越南生猪价格｜南部｜2026-08-02</t>
+          <t>越南生猪价格｜南部｜2026-08-03</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1404,7 @@
       <c r="C5" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D5" s="9" t="n"/>
+      <c r="D5" s="8" t="n"/>
       <c r="E5" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1443,7 +1425,7 @@
       <c r="C6" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D6" s="9" t="n"/>
+      <c r="D6" s="8" t="n"/>
       <c r="E6" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1464,7 +1446,7 @@
       <c r="C7" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D7" s="9" t="n"/>
+      <c r="D7" s="8" t="n"/>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1485,12 +1467,10 @@
       <c r="C8" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D8" s="8" t="n">
-        <v>-1000</v>
-      </c>
+      <c r="D8" s="8" t="n"/>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>下降</t>
+          <t>稳定</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1488,7 @@
       <c r="C9" s="6" t="n">
         <v>60000</v>
       </c>
-      <c r="D9" s="9" t="n"/>
+      <c r="D9" s="8" t="n"/>
       <c r="E9" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1529,7 +1509,7 @@
       <c r="C10" s="6" t="n">
         <v>62000</v>
       </c>
-      <c r="D10" s="9" t="n"/>
+      <c r="D10" s="8" t="n"/>
       <c r="E10" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1550,7 +1530,7 @@
       <c r="C11" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D11" s="9" t="n"/>
+      <c r="D11" s="8" t="n"/>
       <c r="E11" s="5" t="inlineStr">
         <is>
           <t>稳定</t>
@@ -1571,7 +1551,7 @@
       <c r="C12" s="6" t="n">
         <v>61000</v>
       </c>
-      <c r="D12" s="9" t="n"/>
+      <c r="D12" s="8" t="n"/>
       <c r="E12" s="5" t="inlineStr">
         <is>
           <t>稳定</t>

</xml_diff>